<commit_message>
Fixed templates, spelling, lowercase, spaces in view and the last coverage pages
</commit_message>
<xml_diff>
--- a/static/Files/Template - Cluster - Numeric.xlsx
+++ b/static/Files/Template - Cluster - Numeric.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcs839\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcs839\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C465ED-9EB2-4851-8E8A-F291E09AA39F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D64F6A-18CE-4F6C-BA8A-F8FF6D8ABC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4360,6 +4360,14 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="21">
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -4611,14 +4619,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border outline="0">
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -4655,12 +4655,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A6C002E2-BB37-4C86-B7CA-6AC21ECCFF45}" name="ClusterTable" displayName="ClusterTable" ref="A1:D806" totalsRowShown="0" headerRowBorderDxfId="20" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A6C002E2-BB37-4C86-B7CA-6AC21ECCFF45}" name="ClusterTable" displayName="ClusterTable" ref="A1:D805" totalsRowShown="0" headerRowBorderDxfId="20" tableBorderDxfId="19">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{73FDEE34-CD20-4B8C-863F-078A12833161}" name="GPCRs_x000a_(Gene or Uniprot name)" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{0683A298-F68D-4C14-A78A-80F39A293AD9}" name="Add numbers_x000a_(Visualized as Gradient _x000a_of one or two colors)" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{EDF0D28B-B001-4AAD-A09F-C16FDBA10C01}" name="Optional: _x000a_Add Numbers _x000a_(Spatial positioning)" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{E9EFDE34-373F-4AB6-A635-F486FD348B4A}" name="Info / error" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{73FDEE34-CD20-4B8C-863F-078A12833161}" name="GPCRs_x000a_(Gene or Uniprot name)" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{0683A298-F68D-4C14-A78A-80F39A293AD9}" name="Add numbers_x000a_(Visualized as Gradient _x000a_of one or two colors)" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{EDF0D28B-B001-4AAD-A09F-C16FDBA10C01}" name="Optional: _x000a_Add Numbers _x000a_(Spatial positioning)" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{E9EFDE34-373F-4AB6-A635-F486FD348B4A}" name="Info / error" dataDxfId="16">
       <calculatedColumnFormula>IF(A2="",
     IF(COUNTA(B2:C2)&gt;0, "You need to select a GPCR.", ""),
     IF(SUM(
@@ -4694,17 +4694,17 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8F6FC1CD-B142-4F94-8C86-4E8AE110AD29}" name="ReceptorData" displayName="ReceptorData" ref="A1:E805" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8F6FC1CD-B142-4F94-8C86-4E8AE110AD29}" name="ReceptorData" displayName="ReceptorData" ref="A1:E805" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:E805" xr:uid="{8F6FC1CD-B142-4F94-8C86-4E8AE110AD29}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E805">
     <sortCondition ref="E1:E1048575"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7EFCA3FF-1755-4B34-A3E6-68FEC263B14E}" name="GPCRs_x000a_(UniProt)" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{0E4AA618-9775-4FA6-BD46-12A7F5D47E89}" name="GPCRs_x000a_(Gene name)" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{BEF0682F-C1C7-43DC-B2F7-E432261E366A}" name="Receptor family" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{D2ED2812-3409-4307-924A-E866BD70C70B}" name="Ligand type" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{33ED79F7-22B3-4243-BABD-052ACEAEF199}" name="Class" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{7EFCA3FF-1755-4B34-A3E6-68FEC263B14E}" name="GPCRs_x000a_(UniProt)" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{0E4AA618-9775-4FA6-BD46-12A7F5D47E89}" name="GPCRs_x000a_(Gene name)" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{BEF0682F-C1C7-43DC-B2F7-E432261E366A}" name="Receptor family" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{D2ED2812-3409-4307-924A-E866BD70C70B}" name="Ligand type" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{33ED79F7-22B3-4243-BABD-052ACEAEF199}" name="Class" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4974,7 +4974,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F26E749E-D107-4E22-80D8-C6EBAA01D602}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:D806"/>
+  <dimension ref="A1:D805"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.6328125" customWidth="1"/>
@@ -32333,70 +32333,36 @@
         <v/>
       </c>
     </row>
-    <row r="806" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A806" s="8"/>
-      <c r="B806" s="10"/>
-      <c r="C806" s="10"/>
-      <c r="D806" s="10" t="str">
-        <f>IF(A806="",
-    IF(COUNTA(B806:C806)&gt;0, "You need to select a GPCR.", ""),
-    IF(SUM(
-        COUNTIF(ReceptorData[GPCRs
-(UniProt)], A806),
-        COUNTIF(ReceptorData[GPCRs
-(Gene name)], A806)
-    )=0,
-        "Invalid GPCR (Try to take a look at the 'GPCR lookup table' Sheet).",
-        IF(AND(C806="", A806&lt;&gt;"", B806=""),
-            "Need a number in column B.",
-            IF(AND(C806&lt;&gt;"", B806=""),
-                "Need a number in column B together with spatial position.",
-                IF(AND(NOT(ISNUMBER(B806))),
-                    "Non-numeric value detected in Column B.",
-                    IF(AND(C806&lt;&gt;"", NOT(ISNUMBER(C806))),
-                        "Non-numeric value detected in Column C.",
-                        IF(AND(A806&lt;&gt;"", ISNUMBER(B806), OR(C806="", ISNUMBER(C806))),
-                            "Data is correctly formatted.",
-                            "")
-                    )
-                )
-            )
-        )
-    )
-)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="D2:D806">
-    <cfRule type="expression" dxfId="7" priority="1">
+  <conditionalFormatting sqref="D2:D805">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>D2="You need to select a GPCR."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>D2="Invalid GPCR (Try to take a look at the 'GPCR lookup table' Sheet)."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>D2="Non-numeric value detected in Column C."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>D2="Non-numeric value detected in Column B."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>D2="Non-numeric value detected in Column B and C."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="6">
+    <cfRule type="expression" dxfId="3" priority="6">
       <formula>D2="Need a number in column B together with spatial position."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="7">
+    <cfRule type="expression" dxfId="2" priority="7">
       <formula>D2="Data is correctly formatted."</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="1" priority="8">
       <formula>D2="Need a number in column B."</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A807:A1048576" xr:uid="{86A6EA20-CE03-4F82-9E14-B7B23BAD19B1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A806:A1048576" xr:uid="{86A6EA20-CE03-4F82-9E14-B7B23BAD19B1}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>